<commit_message>
add excel that works in progress
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/DataStore.xlsx
+++ b/tests/resources/test_data/DataStore.xlsx
@@ -8,9 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="_pattern" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2026-05-13_09_37_30" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026-05-13_09_39_05" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2026-05-13_09_39_16" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-05-13_09_46_23" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
@@ -349,153 +347,29 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Some rule name 1</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Line,1</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Line, 1</t>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Line before 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Line after 1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Some rule name 2</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Line,2</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Line, 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="12.75" customHeight="1" s="3"/>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="6.14" customWidth="1" style="2" min="1" max="1"/>
-    <col width="7.88" customWidth="1" style="2" min="2" max="2"/>
-    <col width="5.79" customWidth="1" style="2" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="12.75" customHeight="1" s="3">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">before  </t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">after </t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Some rule name 1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Line before 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="12.75" customHeight="1" s="3"/>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="6.14" customWidth="1" style="2" min="1" max="1"/>
-    <col width="7.88" customWidth="1" style="2" min="2" max="2"/>
-    <col width="5.79" customWidth="1" style="2" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="12.75" customHeight="1" s="3">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">before  </t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">after </t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Some rule name 1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Line before 1</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Line after 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Some rule name 2</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Line before 2</t>
         </is>

</xml_diff>

<commit_message>
add excel that works in progress 2
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/DataStore.xlsx
+++ b/tests/resources/test_data/DataStore.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="_pattern" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2026-05-13_09_46_23" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-05-13_10_01_17" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
@@ -321,7 +321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6.14" customWidth="1" style="2" min="1" max="1"/>
@@ -380,6 +380,125 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Some rule name 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Line before 3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Line after 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Some rule name 4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Line before 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Line after 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Some rule name 5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Line before 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Line after 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Some rule name 6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Line before 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Line after 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Some rule name 7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Line before 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Line after 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Some rule name 8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Line before 8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Line after 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Some rule name 9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Line before 9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Line after 9</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="12.75" customHeight="1" s="3"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
works correctly final tested
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/DataStore.xlsx
+++ b/tests/resources/test_data/DataStore.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="_pattern" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2026-05-14_14_47_26" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026-05-18_10_30_27" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-05-18_10_30_27" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2026-05-20_11_04_46" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>

</xml_diff>

<commit_message>
info from common.py added to every script, README backbone done
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/DataStore.xlsx
+++ b/tests/resources/test_data/DataStore.xlsx
@@ -10,6 +10,8 @@
     <sheet name="_pattern" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2026-05-18_10_30_27" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2026-05-20_11_04_46" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2026-05-21_09_14_44" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026-05-21_09_24_48" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.001"/>
@@ -1118,6 +1120,893 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>rock ’n’ roll</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>rock‘n’roll
+rock' n' roll
+rock’n’roll</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>rock ’n’ roll
+rock ’n’ roll
+rock ’n’ roll</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>English, English (UK), English (US), German (Germany), Spanish</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Guns N’ Roses</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Guns’N’Roses
+Guns n'Roses
+Guns ‘N’ Roses</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Guns N’ Roses
+Guns N’ Roses
+Guns N’ Roses</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Czech (academic rules), Czech (traditional rules), English, English (UK), English (US), German (Germany), Spanish</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Correct form of C. a K. in Czech</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>C.a k.
+C. a k.</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>C.&amp;nbsp;a&amp;nbsp;k.
+C.&amp;nbsp;a&amp;nbsp;k.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Czech (academic rules), Czech (traditional rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Change E followed by apostrophe by È</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>E' (Italian)
+E’ (Italian)
+E` (Italian)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>È (Italian)
+È (Italian)
+È (Italian)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Italian</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ą</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>ę</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>ż</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Ą</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Ę</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Ż</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Convert micro to proper Greek μ if surrounded by Greek letters</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>αµα</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>αμα</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Greek</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="12.75" customHeight="1" s="4">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Convert semicolon to proper Greek ; if placed after any Greek letter</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Άλφα;</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Άλφα;</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Greek</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Convert middot to proper Greek · if placed after any Greek letter</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Άλφα·</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Άλφα·</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Greek</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Convert Ohm to proper Greek Ω if surrounded by Greek letters</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Ωμέγα</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Ωμέγα</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Greek</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Dr or Pr without period</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Dr. François</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Dr&amp;nbsp;François</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>French</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Replace i jacute by iacute jacute iȷ́ –&gt; íȷ́</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>liȷ́n (Dutch)
+lij́n (Dutch)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>líȷ́n (Dutch)
+líȷ́n (Dutch)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Replace I Jacute by Iacute Jacute IJ́ –&gt; ÍJ́</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>LIJ́N (Dutch)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>LÍJ́N (Dutch)</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Dutch</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Nonbreaking spaces in N. de la A.</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>N. de la A.</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>N. de la A.</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Nonbreaking spaces in a D. g.</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>a D. g. (Spanish)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>a D. g. (Spanish)</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Nonbreaking spaces in a s. e. u o.</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>s. e. u o.</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>s. e. u o.</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Correct Hungarian un. to ún.</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Ez az un. minimalista stílus</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Ez az ún. minimalista stílus</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Hungarian</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Correct form of et al.</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Author et all
+Author et al
+Author et all.</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Author et&amp;nbsp;al.
+Author et&amp;nbsp;al.
+Author et&amp;nbsp;al.</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Czech (academic rules), Czech (traditional rules), English (UK), English (US)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Correct form of ș U+0219</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Romanian</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Correct form of ț U+021B</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Romanian</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Correct form of Ș U+0218</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Romanian</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Correct form of Ț U+021A</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Romanian</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Use precomposed glyph á</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Czech (academic rules), Czech (traditional rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Use precomposed glyph Á</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Czech (academic rules), Czech (traditional rules), Slovak</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Use precomposed glyph ć</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Czech (academic rules), Czech (traditional rules), Polish</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Use precomposed glyph Ć</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Czech (academic rules), Czech (traditional rules), Polish, Slovenian</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="8.52" customWidth="1" style="3" min="1" max="1"/>
+    <col width="6.02" customWidth="1" style="3" min="2" max="2"/>
+    <col width="10.2" customWidth="1" style="3" min="3" max="3"/>
+    <col width="8.800000000000001" customWidth="1" style="3" min="4" max="4"/>
+    <col width="10.33" customWidth="1" style="3" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="12.75" customHeight="1" s="4">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id          </t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>text before</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>text after</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">languages </t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Some rule name 1</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Line before 1</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Line  Line Line  after 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Some rule name 2</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Line before 2</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Line  Line Line  after 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Some rule name 3</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Line before 3</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Line  Line Line  after 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Some rule name 4</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Line before 4</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Line  Line Line  after 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="12.75" customHeight="1" s="4"/>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="8.52" customWidth="1" style="3" min="1" max="1"/>
+    <col width="6.02" customWidth="1" style="3" min="2" max="2"/>
+    <col width="10.2" customWidth="1" style="3" min="3" max="3"/>
+    <col width="8.800000000000001" customWidth="1" style="3" min="4" max="4"/>
+    <col width="10.33" customWidth="1" style="3" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="12.75" customHeight="1" s="4">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id          </t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>text before</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>text after</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">languages </t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>41</t>

</xml_diff>